<commit_message>
Updated existing test cases and added comments.
</commit_message>
<xml_diff>
--- a/TestData/DataDriven.xlsx
+++ b/TestData/DataDriven.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2445" windowWidth="16335" windowHeight="3825" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="2445" windowWidth="15645" windowHeight="6615" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -15,6 +15,7 @@
     <sheet name="Very Strong pwd" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A1:K20"/>
 </workbook>
 </file>
 
@@ -1012,63 +1013,63 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>63</v>
       </c>

</xml_diff>